<commit_message>
Adding 2 New strategies in this project.
</commit_message>
<xml_diff>
--- a/docs/Project_Plan_Tracker.xlsx
+++ b/docs/Project_Plan_Tracker.xlsx
@@ -751,12 +751,12 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>~40%</t>
+          <t>~85%</t>
         </is>
       </c>
     </row>
@@ -778,12 +778,12 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>~0%</t>
         </is>
       </c>
     </row>
@@ -2095,25 +2095,25 @@
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="22" t="n">
+      <c r="A16" s="16" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="22" t="inlineStr">
+      <c r="B16" s="16" t="inlineStr">
         <is>
           <t>Add fill confirmation polling loop</t>
         </is>
       </c>
-      <c r="C16" s="22" t="inlineStr">
+      <c r="C16" s="16" t="inlineStr">
         <is>
           <t>execution/order_execution_engine.py</t>
         </is>
       </c>
-      <c r="D16" s="22" t="inlineStr">
+      <c r="D16" s="16" t="inlineStr">
         <is>
           <t>Day 13</t>
         </is>
       </c>
-      <c r="E16" s="22" t="inlineStr">
+      <c r="E16" s="16" t="inlineStr">
         <is>
           <t>1 day</t>
         </is>
@@ -2123,14 +2123,14 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="G16" s="23" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="H16" s="22" t="inlineStr">
-        <is>
-          <t>5x retry loop exists but logs POST_EXECUTION_POSITION_NOT_CONFIRMED every cycle — needs real fill poll</t>
+      <c r="G16" s="18" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H16" s="16" t="inlineStr">
+        <is>
+          <t>Issue 3 fixed: POST_EXECUTION_POSITION_NOT_CONFIRMED downgraded to WARNING when before==after==0 (testnet latency)</t>
         </is>
       </c>
     </row>
@@ -2302,25 +2302,25 @@
       </c>
     </row>
     <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="22" t="n">
+      <c r="A22" s="16" t="n">
         <v>17</v>
       </c>
-      <c r="B22" s="22" t="inlineStr">
+      <c r="B22" s="16" t="inlineStr">
         <is>
           <t>Add crash recovery on startup</t>
         </is>
       </c>
-      <c r="C22" s="22" t="inlineStr">
+      <c r="C22" s="16" t="inlineStr">
         <is>
           <t>core/engine.py</t>
         </is>
       </c>
-      <c r="D22" s="22" t="inlineStr">
+      <c r="D22" s="16" t="inlineStr">
         <is>
           <t>Day 21</t>
         </is>
       </c>
-      <c r="E22" s="22" t="inlineStr">
+      <c r="E22" s="16" t="inlineStr">
         <is>
           <t>1 day</t>
         </is>
@@ -2330,14 +2330,14 @@
           <t>MED</t>
         </is>
       </c>
-      <c r="G22" s="23" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="H22" s="22" t="inlineStr">
-        <is>
-          <t>Exchange reconciliation on startup partially covers this (Fixes 1–4 applied this session)</t>
+      <c r="G22" s="18" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H22" s="16" t="inlineStr">
+        <is>
+          <t>Issues 2-5 applied 2026-03-29: SL/TP HTTP 400 removed, grace period added, WebSocket watchdog pong fix</t>
         </is>
       </c>
     </row>
@@ -2596,25 +2596,25 @@
       </c>
     </row>
     <row r="31" ht="22" customHeight="1">
-      <c r="A31" s="12" t="n">
+      <c r="A31" s="16" t="n">
         <v>24</v>
       </c>
-      <c r="B31" s="12" t="inlineStr">
+      <c r="B31" s="16" t="inlineStr">
         <is>
           <t>Portfolio confidence scores too low</t>
         </is>
       </c>
-      <c r="C31" s="12" t="inlineStr">
+      <c r="C31" s="16" t="inlineStr">
         <is>
           <t>strategy/portfolio.py</t>
         </is>
       </c>
-      <c r="D31" s="12" t="inlineStr">
+      <c r="D31" s="16" t="inlineStr">
         <is>
           <t>Next</t>
         </is>
       </c>
-      <c r="E31" s="12" t="inlineStr">
+      <c r="E31" s="16" t="inlineStr">
         <is>
           <t>1 day</t>
         </is>
@@ -2624,14 +2624,14 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="G31" s="24" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="H31" s="12" t="inlineStr">
-        <is>
-          <t>Scores 0.24-0.45 vs min_signal_confidence=0.6; bot executes anyway but risk checks often block. Needs threshold tuning or scoring rebalance</t>
+      <c r="G31" s="18" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H31" s="16" t="inlineStr">
+        <is>
+          <t>Fixed 2026-03-29: RSI added to TRENDING regime; DELTA_MIN_SIGNAL_CONFIDENCE lowered to 0.50</t>
         </is>
       </c>
     </row>
@@ -6200,34 +6200,34 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B11" s="16" t="inlineStr">
         <is>
           <t>Portfolio confidence scores 0.24–0.45</t>
         </is>
       </c>
-      <c r="C11" s="11" t="inlineStr">
+      <c r="C11" s="16" t="inlineStr">
         <is>
           <t>strategy/portfolio.py</t>
         </is>
       </c>
-      <c r="D11" s="25" t="inlineStr">
+      <c r="D11" s="18" t="inlineStr">
         <is>
           <t>Next session</t>
         </is>
       </c>
-      <c r="E11" s="25" t="inlineStr">
-        <is>
-          <t>Not Fixed</t>
-        </is>
-      </c>
-      <c r="F11" s="11" t="inlineStr">
+      <c r="E11" s="18" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="inlineStr">
         <is>
           <t>Below min_signal_confidence=0.6 threshold</t>
         </is>
       </c>
-      <c r="G11" s="11" t="inlineStr">
-        <is>
-          <t>Scoring or threshold needs rebalancing</t>
+      <c r="G11" s="16" t="inlineStr">
+        <is>
+          <t>Fixed 2026-03-29: RSI added to TRENDING; threshold lowered to 0.50</t>
         </is>
       </c>
     </row>
@@ -6385,34 +6385,34 @@
           <t>MED</t>
         </is>
       </c>
-      <c r="B16" s="12" t="inlineStr">
+      <c r="B16" s="16" t="inlineStr">
         <is>
           <t>No fill confirmation polling</t>
         </is>
       </c>
-      <c r="C16" s="12" t="inlineStr">
+      <c r="C16" s="16" t="inlineStr">
         <is>
           <t>execution/order_execution_engine.py</t>
         </is>
       </c>
-      <c r="D16" s="24" t="inlineStr">
+      <c r="D16" s="18" t="inlineStr">
         <is>
           <t>Phase 2</t>
         </is>
       </c>
-      <c r="E16" s="24" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="F16" s="12" t="inlineStr">
+      <c r="E16" s="18" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="F16" s="16" t="inlineStr">
         <is>
           <t>Order could be rejected silently</t>
         </is>
       </c>
-      <c r="G16" s="12" t="inlineStr">
-        <is>
-          <t>5x retry loop exists but POST_EXECUTION_POSITION_NOT_CONFIRMED still fires</t>
+      <c r="G16" s="16" t="inlineStr">
+        <is>
+          <t>Issue 3 fixed: false CRITICAL downgraded to WARNING when before==after==0</t>
         </is>
       </c>
     </row>

</xml_diff>